<commit_message>
New Changes in NRHS
</commit_message>
<xml_diff>
--- a/NRCS/Requirements/NRCS_School_Timetable_5Jul2026.xlsx
+++ b/NRCS/Requirements/NRCS_School_Timetable_5Jul2026.xlsx
@@ -5,23 +5,24 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanwin/Documents/NallamSchools/NRCS/Time Table/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanwin/Documents/GitHub/School_TimeTable/NRCS/Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE4EAEC8-2E55-B745-8D04-2E44348ED7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{822574CB-5C9D-B84F-8386-9030E8CB6F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Class Time Table" sheetId="1" r:id="rId1"/>
-    <sheet name="Teacher Time Table" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
+    <sheet name="Teacher Time Table" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1506" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1661" uniqueCount="238">
   <si>
     <t>TEACHER: BHAVANI</t>
   </si>
@@ -767,6 +768,35 @@
   </si>
   <si>
     <t>Class 1 to 8 (KARATE)</t>
+  </si>
+  <si>
+    <t>Swathi(Hin)</t>
+  </si>
+  <si>
+    <t>Sai Lakshmi(Hin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naga mani
+</t>
+  </si>
+  <si>
+    <t>Bhavani</t>
+  </si>
+  <si>
+    <t>Riya(Hin)</t>
+  </si>
+  <si>
+    <t>Gowtham</t>
+  </si>
+  <si>
+    <t>Bheema
+(PHY/Chem))</t>
+  </si>
+  <si>
+    <t>Sonu(Eng)</t>
+  </si>
+  <si>
+    <t>Ravi(Eng-Greammer</t>
   </si>
 </sst>
 </file>
@@ -920,7 +950,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -982,11 +1012,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1050,6 +1089,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3423,6 +3472,765 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E7D8A15-BABD-484A-A51A-77DB1450FE13}">
+  <dimension ref="A1:N49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A3" s="19"/>
+      <c r="B3" s="2">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="M3" s="26" t="s">
+        <v>233</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A4" s="19"/>
+      <c r="B4" s="2">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="N4" s="26" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A5" s="19"/>
+      <c r="B5" s="2">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A6" s="19"/>
+      <c r="B6" s="2">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="N6" s="27" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A7" s="19"/>
+      <c r="B7" s="2">
+        <v>6</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="N7" s="27"/>
+    </row>
+    <row r="8" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A8" s="19"/>
+      <c r="B8" s="2">
+        <v>7</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="M8" s="27" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+      <c r="A9" s="20"/>
+      <c r="B9" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="M9" s="7"/>
+      <c r="N9" s="27" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A10" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="B10" s="2">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A11" s="19"/>
+      <c r="B11" s="2">
+        <v>2</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A12" s="19"/>
+      <c r="B12" s="2">
+        <v>3</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A13" s="19"/>
+      <c r="B13" s="2">
+        <v>4</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A14" s="19"/>
+      <c r="B14" s="2">
+        <v>5</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A15" s="19"/>
+      <c r="B15" s="2">
+        <v>6</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="A16" s="19"/>
+      <c r="B16" s="2">
+        <v>7</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A17" s="20"/>
+      <c r="B17" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A18" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B18" s="2">
+        <v>1</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A19" s="19"/>
+      <c r="B19" s="2">
+        <v>2</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A20" s="19"/>
+      <c r="B20" s="2">
+        <v>3</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A21" s="19"/>
+      <c r="B21" s="2">
+        <v>4</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A22" s="19"/>
+      <c r="B22" s="2">
+        <v>5</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A23" s="19"/>
+      <c r="B23" s="2">
+        <v>6</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A24" s="19"/>
+      <c r="B24" s="2">
+        <v>7</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A25" s="20"/>
+      <c r="B25" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A26" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="B26" s="2">
+        <v>1</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A27" s="19"/>
+      <c r="B27" s="2">
+        <v>2</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A28" s="19"/>
+      <c r="B28" s="2">
+        <v>3</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A29" s="19"/>
+      <c r="B29" s="2">
+        <v>4</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A30" s="19"/>
+      <c r="B30" s="2">
+        <v>5</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A31" s="19"/>
+      <c r="B31" s="2">
+        <v>6</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A32" s="19"/>
+      <c r="B32" s="2">
+        <v>7</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A33" s="20"/>
+      <c r="B33" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A34" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="B34" s="2">
+        <v>1</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A35" s="19"/>
+      <c r="B35" s="2">
+        <v>2</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A36" s="19"/>
+      <c r="B36" s="2">
+        <v>3</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A37" s="19"/>
+      <c r="B37" s="2">
+        <v>4</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A38" s="19"/>
+      <c r="B38" s="2">
+        <v>5</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A39" s="19"/>
+      <c r="B39" s="2">
+        <v>6</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A40" s="19"/>
+      <c r="B40" s="2">
+        <v>7</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A41" s="20"/>
+      <c r="B41" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A42" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="B42" s="2">
+        <v>1</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A43" s="19"/>
+      <c r="B43" s="2">
+        <v>2</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A44" s="19"/>
+      <c r="B44" s="2">
+        <v>3</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A45" s="19"/>
+      <c r="B45" s="2">
+        <v>4</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A46" s="19"/>
+      <c r="B46" s="2">
+        <v>5</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A47" s="19"/>
+      <c r="B47" s="2">
+        <v>6</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="26" x14ac:dyDescent="0.2">
+      <c r="A48" s="19"/>
+      <c r="B48" s="2">
+        <v>7</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="20"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:A9"/>
+    <mergeCell ref="A10:A17"/>
+    <mergeCell ref="A18:A25"/>
+    <mergeCell ref="A26:A33"/>
+    <mergeCell ref="A34:A41"/>
+    <mergeCell ref="A42:A49"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -7308,14 +8116,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A48:I48"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="A183:I183"/>
-    <mergeCell ref="A174:I174"/>
-    <mergeCell ref="A75:I75"/>
-    <mergeCell ref="A84:I84"/>
-    <mergeCell ref="A66:I66"/>
-    <mergeCell ref="A120:I120"/>
     <mergeCell ref="A201:I201"/>
     <mergeCell ref="A138:I138"/>
     <mergeCell ref="A1:I1"/>
@@ -7332,6 +8132,14 @@
     <mergeCell ref="A111:I111"/>
     <mergeCell ref="A102:I102"/>
     <mergeCell ref="A39:I39"/>
+    <mergeCell ref="A48:I48"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A183:I183"/>
+    <mergeCell ref="A174:I174"/>
+    <mergeCell ref="A75:I75"/>
+    <mergeCell ref="A84:I84"/>
+    <mergeCell ref="A66:I66"/>
+    <mergeCell ref="A120:I120"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="63" fitToHeight="10" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>